<commit_message>
feat: add sql questions
</commit_message>
<xml_diff>
--- a/storage/initdata/ごみ分別_initdata.xlsx
+++ b/storage/initdata/ごみ分別_initdata.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -4003,6 +4003,7 @@
         <sz val="12"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
       </rPr>
       <t xml:space="preserve"> </t>
     </r>
@@ -4023,7 +4024,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -4048,6 +4049,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="128"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">

</xml_diff>